<commit_message>
feat: auto-seed demo directories on startup
</commit_message>
<xml_diff>
--- a/sample_documents/sample_worklog.xlsx
+++ b/sample_documents/sample_worklog.xlsx
@@ -469,10 +469,8 @@
           <t>Электромонтажные работы</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>8 часов</t>
-        </is>
+      <c r="E2" t="n">
+        <v>8</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>

</xml_diff>